<commit_message>
Cap nhat giao dien va du lieu he thong den chieu 08-09
</commit_message>
<xml_diff>
--- a/media/exports/Danh_Sach_Dang_Ky_Tu_Van_SHK.xlsx
+++ b/media/exports/Danh_Sach_Dang_Ky_Tu_Van_SHK.xlsx
@@ -502,7 +502,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Thời gian cập nhật: 27/08/2026 13:33:15</t>
+          <t>Thời gian cập nhật: 28/08/2026 10:34:04</t>
         </is>
       </c>
     </row>
@@ -555,32 +555,33 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Nguyen Van A</t>
+          <t>Nguyễn Minh Đức</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>0912345678</t>
+          <t>0389592301</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>vana@gmail.com</t>
+          <t>minhducnguyenforwork@gmail.com</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Cong ty Xay dung A</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Can tu van 500 bao keo</t>
+          <t>Khu vực: Hưng Yên / Trực tuyến
+Nhu cầu: E-Catalog &amp; Tài liệu kỹ thuật SHK Mortar</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>27/08/2026 06:33</t>
+          <t>28/08/2026 03:34</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">

</xml_diff>